<commit_message>
Update LoL data 2026-08-11
</commit_message>
<xml_diff>
--- a/data/excel/lol_report.xlsx
+++ b/data/excel/lol_report.xlsx
@@ -20,8 +20,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'キュー別'!$A$1:$L$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'チャンピオン別'!$A$1:$L$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'SUPチャンピオン別'!$A$1:$L$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'試合履歴'!$A$1:$V$390</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'レビュー'!$A$1:$P$390</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'試合履歴'!$A$1:$V$391</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'レビュー'!$A$1:$P$391</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -532,14 +532,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>対象期間：2026-01-09 23:36:27 ～ 2026-08-10 23:30:12</t>
+          <t>対象期間：2026-01-05 23:21:47 ～ 2026-08-10 23:30:12</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>出力日時：2026-08-11 00:38:07</t>
+          <t>出力日時：2026-08-11 12:05:15</t>
         </is>
       </c>
     </row>
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="7">
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="9">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>0.4755784061696658</v>
+        <v>0.4743589743589743</v>
       </c>
     </row>
     <row r="10">
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>1.704370179948586</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="11">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>5.372750642673521</v>
+        <v>5.371794871794871</v>
       </c>
     </row>
     <row r="12">
@@ -617,7 +617,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>8.9280205655527</v>
+        <v>8.928205128205128</v>
       </c>
     </row>
     <row r="13">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>59.89717223650386</v>
+        <v>59.83333333333334</v>
       </c>
     </row>
     <row r="15">
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>2.036786632390745</v>
+        <v>2.034538461538463</v>
       </c>
     </row>
     <row r="16">
@@ -659,7 +659,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>57.43444730077121</v>
+        <v>57.4025641025641</v>
       </c>
     </row>
     <row r="17">
@@ -669,7 +669,7 @@
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>1.849177377892031</v>
+        <v>1.848282051282051</v>
       </c>
     </row>
     <row r="19">
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="21">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="23">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>0.5065359477124183</v>
+        <v>0.504885993485342</v>
       </c>
     </row>
     <row r="24">
@@ -726,7 +726,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>1.477124183006536</v>
+        <v>1.472312703583062</v>
       </c>
     </row>
     <row r="25">
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>5.202614379084967</v>
+        <v>5.201954397394137</v>
       </c>
     </row>
     <row r="26">
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>9.803921568627452</v>
+        <v>9.801302931596091</v>
       </c>
     </row>
     <row r="27">
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>36.58823529411764</v>
+        <v>36.58306188925081</v>
       </c>
     </row>
     <row r="29">
@@ -778,7 +778,7 @@
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>1.256895424836601</v>
+        <v>1.25657980456026</v>
       </c>
     </row>
     <row r="30">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>64.7516339869281</v>
+        <v>64.68729641693811</v>
       </c>
     </row>
     <row r="31">
@@ -798,7 +798,7 @@
         </is>
       </c>
       <c r="B31" s="8" t="n">
-        <v>2.083202614379085</v>
+        <v>2.08130293159609</v>
       </c>
     </row>
   </sheetData>
@@ -821,7 +821,7 @@
     <col width="5" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
     <col width="6" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
@@ -898,25 +898,25 @@
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C2" s="4" t="n">
         <v>155</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.5065359477124183</v>
+        <v>0.504885993485342</v>
       </c>
       <c r="F2" s="6" t="n">
-        <v>1.477124183006536</v>
+        <v>1.472312703583062</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>5.202614379084967</v>
+        <v>5.201954397394137</v>
       </c>
       <c r="H2" s="6" t="n">
-        <v>9.803921568627452</v>
+        <v>9.801302931596091</v>
       </c>
       <c r="I2" s="7" t="inlineStr">
         <is>
@@ -924,13 +924,13 @@
         </is>
       </c>
       <c r="J2" s="6" t="n">
-        <v>1.256895424836601</v>
+        <v>1.25657980456026</v>
       </c>
       <c r="K2" s="6" t="n">
-        <v>64.7516339869281</v>
+        <v>64.68729641693811</v>
       </c>
       <c r="L2" s="8" t="n">
-        <v>2.083202614379085</v>
+        <v>2.08130293159609</v>
       </c>
     </row>
     <row r="3">
@@ -1050,7 +1050,7 @@
         </is>
       </c>
       <c r="J5" s="6" t="n">
-        <v>4.924590163934426</v>
+        <v>4.924590163934425</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>32.32786885245902</v>
@@ -1133,7 +1133,7 @@
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="6" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
     <col width="19" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
   </cols>
@@ -1233,7 +1233,7 @@
         </is>
       </c>
       <c r="J2" s="6" t="n">
-        <v>2.226996805111821</v>
+        <v>2.226996805111822</v>
       </c>
       <c r="K2" s="6" t="n">
         <v>54.02875399361022</v>
@@ -1249,25 +1249,25 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C3" s="4" t="n">
         <v>32</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0.4210526315789473</v>
+        <v>0.4155844155844156</v>
       </c>
       <c r="F3" s="6" t="n">
-        <v>1.157894736842105</v>
+        <v>1.142857142857143</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>5.828947368421052</v>
+        <v>5.818181818181818</v>
       </c>
       <c r="H3" s="6" t="n">
-        <v>10.07894736842105</v>
+        <v>10.06493506493507</v>
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
@@ -1275,13 +1275,13 @@
         </is>
       </c>
       <c r="J3" s="6" t="n">
-        <v>1.253421052631579</v>
+        <v>1.252207792207792</v>
       </c>
       <c r="K3" s="6" t="n">
-        <v>71.46052631578948</v>
+        <v>71.11688311688312</v>
       </c>
       <c r="L3" s="8" t="n">
-        <v>2.231447368421053</v>
+        <v>2.221948051948053</v>
       </c>
     </row>
   </sheetData>
@@ -1458,7 +1458,7 @@
         </is>
       </c>
       <c r="J3" s="6" t="n">
-        <v>1.490185185185185</v>
+        <v>1.490185185185186</v>
       </c>
       <c r="K3" s="6" t="n">
         <v>62.64814814814815</v>
@@ -1516,25 +1516,25 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>16</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.4102564102564102</v>
+        <v>0.4</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.7948717948717948</v>
+        <v>0.775</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>5.153846153846154</v>
+        <v>5.15</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>7.17948717948718</v>
+        <v>7.225</v>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
@@ -1542,13 +1542,13 @@
         </is>
       </c>
       <c r="J5" s="6" t="n">
-        <v>1.232820512820513</v>
+        <v>1.231</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>53.97435897435897</v>
+        <v>53.75</v>
       </c>
       <c r="L5" s="8" t="n">
-        <v>1.871025641025641</v>
+        <v>1.86175</v>
       </c>
     </row>
     <row r="6">
@@ -1584,7 +1584,7 @@
         </is>
       </c>
       <c r="J6" s="6" t="n">
-        <v>5.148285714285715</v>
+        <v>5.148285714285714</v>
       </c>
       <c r="K6" s="6" t="n">
         <v>34.6</v>
@@ -1800,7 +1800,7 @@
         <v>25.625</v>
       </c>
       <c r="L11" s="8" t="n">
-        <v>0.85625</v>
+        <v>0.8562500000000001</v>
       </c>
     </row>
     <row r="12">
@@ -2004,7 +2004,7 @@
         </is>
       </c>
       <c r="J16" s="6" t="n">
-        <v>5.050000000000001</v>
+        <v>5.05</v>
       </c>
       <c r="K16" s="6" t="n">
         <v>16.25</v>
@@ -2833,25 +2833,25 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>16</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.4102564102564102</v>
+        <v>0.4</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.7948717948717948</v>
+        <v>0.775</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>5.153846153846154</v>
+        <v>5.15</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>7.17948717948718</v>
+        <v>7.225</v>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
@@ -2859,13 +2859,13 @@
         </is>
       </c>
       <c r="J5" s="6" t="n">
-        <v>1.232820512820513</v>
+        <v>1.231</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>53.97435897435897</v>
+        <v>53.75</v>
       </c>
       <c r="L5" s="8" t="n">
-        <v>1.871025641025641</v>
+        <v>1.86175</v>
       </c>
     </row>
     <row r="6">
@@ -3266,7 +3266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V390"/>
+  <dimension ref="A1:V391"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -34525,8 +34525,88 @@
         </is>
       </c>
     </row>
+    <row r="391">
+      <c r="A391" s="7" t="inlineStr">
+        <is>
+          <t>2026-01-05 23:21:47</t>
+        </is>
+      </c>
+      <c r="B391" s="7" t="inlineStr">
+        <is>
+          <t>ランク(ソロ/デュオ)</t>
+        </is>
+      </c>
+      <c r="C391" s="12" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D391" s="7" t="inlineStr">
+        <is>
+          <t>SUP</t>
+        </is>
+      </c>
+      <c r="E391" s="7" t="inlineStr">
+        <is>
+          <t>ジャンナ</t>
+        </is>
+      </c>
+      <c r="F391" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G391" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H391" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="I391" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J391" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="K391" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="L391" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="M391" s="6" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="N391" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="O391" s="8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="P391" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q391" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="R391" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="S391" s="11" t="n">
+        <v>6751</v>
+      </c>
+      <c r="T391" s="11" t="n">
+        <v>2219</v>
+      </c>
+      <c r="U391" s="6" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="V391" s="7" t="inlineStr">
+        <is>
+          <t>JP1_556572228</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:V390"/>
+  <autoFilter ref="A1:V391"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -34537,7 +34617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P390"/>
+  <dimension ref="A1:P391"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -58758,8 +58838,70 @@
         </is>
       </c>
     </row>
+    <row r="391">
+      <c r="A391" s="13" t="inlineStr">
+        <is>
+          <t>2026-01-05 23:21:47</t>
+        </is>
+      </c>
+      <c r="B391" s="13" t="inlineStr">
+        <is>
+          <t>ランク</t>
+        </is>
+      </c>
+      <c r="C391" s="13" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D391" s="13" t="inlineStr">
+        <is>
+          <t>SUP</t>
+        </is>
+      </c>
+      <c r="E391" s="13" t="inlineStr">
+        <is>
+          <t>ジャンナ</t>
+        </is>
+      </c>
+      <c r="F391" s="13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G391" s="13" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H391" s="13" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="I391" s="13" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="J391" s="13" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="K391" s="14" t="inlineStr"/>
+      <c r="L391" s="14" t="inlineStr"/>
+      <c r="M391" s="14" t="inlineStr"/>
+      <c r="N391" s="14" t="inlineStr"/>
+      <c r="O391" s="14" t="inlineStr"/>
+      <c r="P391" s="13" t="inlineStr">
+        <is>
+          <t>JP1_556572228</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P390"/>
+  <autoFilter ref="A1:P391"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update LoL data 2026-08-18
</commit_message>
<xml_diff>
--- a/data/excel/lol_report.xlsx
+++ b/data/excel/lol_report.xlsx
@@ -20,8 +20,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'キュー別'!$A$1:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'チャンピオン別'!$A$1:$L$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'SUPチャンピオン別'!$A$1:$L$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'試合履歴'!$A$1:$V$401</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'レビュー'!$A$1:$P$401</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'試合履歴'!$A$1:$V$402</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'レビュー'!$A$1:$P$402</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -532,14 +532,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>対象期間：2026-01-09 23:36:27 ～ 2026-08-18 03:23:21</t>
+          <t>対象期間：2026-01-05 23:21:47 ～ 2026-08-18 03:23:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>出力日時：2026-08-18 03:56:29</t>
+          <t>出力日時：2026-08-18 11:16:46</t>
         </is>
       </c>
     </row>
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="7">
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="9">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>0.475</v>
+        <v>0.4738154613466334</v>
       </c>
     </row>
     <row r="10">
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>1.685</v>
+        <v>1.680798004987531</v>
       </c>
     </row>
     <row r="11">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>5.4275</v>
+        <v>5.42643391521197</v>
       </c>
     </row>
     <row r="12">
@@ -617,7 +617,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>8.967499999999999</v>
+        <v>8.967581047381547</v>
       </c>
     </row>
     <row r="13">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>59.1475</v>
+        <v>59.08728179551122</v>
       </c>
     </row>
     <row r="15">
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>2.00995</v>
+        <v>2.007830423940151</v>
       </c>
     </row>
     <row r="16">
@@ -659,7 +659,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>58.205</v>
+        <v>58.17206982543641</v>
       </c>
     </row>
     <row r="17">
@@ -669,7 +669,7 @@
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>1.8701</v>
+        <v>1.869177057356608</v>
       </c>
     </row>
     <row r="19">
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="21">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="23">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>0.5047318611987381</v>
+        <v>0.5031446540880503</v>
       </c>
     </row>
     <row r="24">
@@ -726,7 +726,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>1.460567823343849</v>
+        <v>1.455974842767296</v>
       </c>
     </row>
     <row r="25">
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>5.277602523659306</v>
+        <v>5.276729559748428</v>
       </c>
     </row>
     <row r="26">
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>9.823343848580441</v>
+        <v>9.820754716981131</v>
       </c>
     </row>
     <row r="27">
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>36.45110410094637</v>
+        <v>36.44654088050314</v>
       </c>
     </row>
     <row r="29">
@@ -778,7 +778,7 @@
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>1.250094637223975</v>
+        <v>1.249811320754717</v>
       </c>
     </row>
     <row r="30">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>65.47003154574132</v>
+        <v>65.40566037735849</v>
       </c>
     </row>
     <row r="31">
@@ -798,7 +798,7 @@
         </is>
       </c>
       <c r="B31" s="8" t="n">
-        <v>2.101482649842271</v>
+        <v>2.099591194968554</v>
       </c>
     </row>
   </sheetData>
@@ -898,25 +898,25 @@
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C2" s="4" t="n">
         <v>160</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.5047318611987381</v>
+        <v>0.5031446540880503</v>
       </c>
       <c r="F2" s="6" t="n">
-        <v>1.460567823343849</v>
+        <v>1.455974842767296</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>5.277602523659306</v>
+        <v>5.276729559748428</v>
       </c>
       <c r="H2" s="6" t="n">
-        <v>9.823343848580441</v>
+        <v>9.820754716981131</v>
       </c>
       <c r="I2" s="7" t="inlineStr">
         <is>
@@ -924,13 +924,13 @@
         </is>
       </c>
       <c r="J2" s="6" t="n">
-        <v>1.250094637223975</v>
+        <v>1.249811320754717</v>
       </c>
       <c r="K2" s="6" t="n">
-        <v>65.47003154574132</v>
+        <v>65.40566037735849</v>
       </c>
       <c r="L2" s="8" t="n">
-        <v>2.101482649842271</v>
+        <v>2.099591194968554</v>
       </c>
     </row>
     <row r="3">
@@ -1050,7 +1050,7 @@
         </is>
       </c>
       <c r="J5" s="6" t="n">
-        <v>4.924590163934426</v>
+        <v>4.924590163934425</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>32.32786885245902</v>
@@ -1128,7 +1128,7 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="5" customWidth="1" min="3" max="3"/>
     <col width="5" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
@@ -1249,25 +1249,25 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C3" s="4" t="n">
         <v>34</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0.4197530864197531</v>
+        <v>0.4146341463414634</v>
       </c>
       <c r="F3" s="6" t="n">
-        <v>1.148148148148148</v>
+        <v>1.134146341463415</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>5.987654320987654</v>
+        <v>5.975609756097561</v>
       </c>
       <c r="H3" s="6" t="n">
-        <v>10.04938271604938</v>
+        <v>10.03658536585366</v>
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
@@ -1275,13 +1275,13 @@
         </is>
       </c>
       <c r="J3" s="6" t="n">
-        <v>1.236296296296296</v>
+        <v>1.235365853658536</v>
       </c>
       <c r="K3" s="6" t="n">
-        <v>71.80246913580247</v>
+        <v>71.47560975609755</v>
       </c>
       <c r="L3" s="8" t="n">
-        <v>2.246666666666667</v>
+        <v>2.237560975609757</v>
       </c>
     </row>
     <row r="4">
@@ -1558,25 +1558,25 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>16</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.4</v>
+        <v>0.3902439024390244</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.825</v>
+        <v>0.8048780487804879</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>5.225</v>
+        <v>5.219512195121951</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>7.05</v>
+        <v>7.097560975609756</v>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
@@ -1584,13 +1584,13 @@
         </is>
       </c>
       <c r="J5" s="6" t="n">
-        <v>1.223</v>
+        <v>1.221463414634147</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>55.55</v>
+        <v>55.29268292682926</v>
       </c>
       <c r="L5" s="8" t="n">
-        <v>1.90925</v>
+        <v>1.899268292682927</v>
       </c>
     </row>
     <row r="6">
@@ -1626,7 +1626,7 @@
         </is>
       </c>
       <c r="J6" s="6" t="n">
-        <v>5.148285714285715</v>
+        <v>5.148285714285714</v>
       </c>
       <c r="K6" s="6" t="n">
         <v>34.6</v>
@@ -1842,7 +1842,7 @@
         <v>25.625</v>
       </c>
       <c r="L11" s="8" t="n">
-        <v>0.85625</v>
+        <v>0.8562500000000001</v>
       </c>
     </row>
     <row r="12">
@@ -2046,7 +2046,7 @@
         </is>
       </c>
       <c r="J16" s="6" t="n">
-        <v>5.050000000000001</v>
+        <v>5.05</v>
       </c>
       <c r="K16" s="6" t="n">
         <v>16.25</v>
@@ -2875,25 +2875,25 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>16</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.4</v>
+        <v>0.3902439024390244</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.825</v>
+        <v>0.8048780487804879</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>5.225</v>
+        <v>5.219512195121951</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>7.05</v>
+        <v>7.097560975609756</v>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
@@ -2901,13 +2901,13 @@
         </is>
       </c>
       <c r="J5" s="6" t="n">
-        <v>1.223</v>
+        <v>1.221463414634147</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>55.55</v>
+        <v>55.29268292682926</v>
       </c>
       <c r="L5" s="8" t="n">
-        <v>1.90925</v>
+        <v>1.899268292682927</v>
       </c>
     </row>
     <row r="6">
@@ -3308,7 +3308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V401"/>
+  <dimension ref="A1:V402"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -35447,8 +35447,88 @@
         </is>
       </c>
     </row>
+    <row r="402">
+      <c r="A402" s="7" t="inlineStr">
+        <is>
+          <t>2026-01-05 23:21:47</t>
+        </is>
+      </c>
+      <c r="B402" s="7" t="inlineStr">
+        <is>
+          <t>ランク(ソロ/デュオ)</t>
+        </is>
+      </c>
+      <c r="C402" s="10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D402" s="7" t="inlineStr">
+        <is>
+          <t>SUP</t>
+        </is>
+      </c>
+      <c r="E402" s="7" t="inlineStr">
+        <is>
+          <t>ジャンナ</t>
+        </is>
+      </c>
+      <c r="F402" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G402" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H402" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="I402" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J402" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="K402" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="L402" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="M402" s="6" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="N402" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="O402" s="8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="P402" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q402" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="R402" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="S402" s="11" t="n">
+        <v>6751</v>
+      </c>
+      <c r="T402" s="11" t="n">
+        <v>2219</v>
+      </c>
+      <c r="U402" s="6" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="V402" s="7" t="inlineStr">
+        <is>
+          <t>JP1_556572228</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:V401"/>
+  <autoFilter ref="A1:V402"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -35459,7 +35539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P401"/>
+  <dimension ref="A1:P402"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -60362,8 +60442,70 @@
         </is>
       </c>
     </row>
+    <row r="402">
+      <c r="A402" s="13" t="inlineStr">
+        <is>
+          <t>2026-01-05 23:21:47</t>
+        </is>
+      </c>
+      <c r="B402" s="13" t="inlineStr">
+        <is>
+          <t>ランク</t>
+        </is>
+      </c>
+      <c r="C402" s="13" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D402" s="13" t="inlineStr">
+        <is>
+          <t>SUP</t>
+        </is>
+      </c>
+      <c r="E402" s="13" t="inlineStr">
+        <is>
+          <t>ジャンナ</t>
+        </is>
+      </c>
+      <c r="F402" s="13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G402" s="13" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H402" s="13" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="I402" s="13" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="J402" s="13" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="K402" s="14" t="inlineStr"/>
+      <c r="L402" s="14" t="inlineStr"/>
+      <c r="M402" s="14" t="inlineStr"/>
+      <c r="N402" s="14" t="inlineStr"/>
+      <c r="O402" s="14" t="inlineStr"/>
+      <c r="P402" s="13" t="inlineStr">
+        <is>
+          <t>JP1_556572228</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P401"/>
+  <autoFilter ref="A1:P402"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update LoL data 2026-08-19
</commit_message>
<xml_diff>
--- a/data/excel/lol_report.xlsx
+++ b/data/excel/lol_report.xlsx
@@ -20,8 +20,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'キュー別'!$A$1:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'チャンピオン別'!$A$1:$L$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'SUPチャンピオン別'!$A$1:$L$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'試合履歴'!$A$1:$V$406</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'レビュー'!$A$1:$P$406</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'試合履歴'!$A$1:$V$407</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'レビュー'!$A$1:$P$407</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -532,14 +532,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>対象期間：2026-01-09 23:36:27 ～ 2026-08-19 00:20:03</t>
+          <t>対象期間：2026-01-05 23:21:47 ～ 2026-08-19 00:20:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>出力日時：2026-08-19 02:54:44</t>
+          <t>出力日時：2026-08-19 11:19:31</t>
         </is>
       </c>
     </row>
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="7">
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="9">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>0.4740740740740741</v>
+        <v>0.4729064039408867</v>
       </c>
     </row>
     <row r="10">
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>1.683950617283951</v>
+        <v>1.679802955665025</v>
       </c>
     </row>
     <row r="11">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>5.432098765432099</v>
+        <v>5.431034482758621</v>
       </c>
     </row>
     <row r="12">
@@ -617,7 +617,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>8.980246913580247</v>
+        <v>8.980295566502463</v>
       </c>
     </row>
     <row r="13">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>58.84691358024691</v>
+        <v>58.78817733990148</v>
       </c>
     </row>
     <row r="15">
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>1.999802469135802</v>
+        <v>1.997733990147784</v>
       </c>
     </row>
     <row r="16">
@@ -659,7 +659,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>58.42962962962963</v>
+        <v>58.39655172413793</v>
       </c>
     </row>
     <row r="17">
@@ -669,7 +669,7 @@
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>1.87841975308642</v>
+        <v>1.877487684729064</v>
       </c>
     </row>
     <row r="19">
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="21">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="23">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>0.5031055900621118</v>
+        <v>0.5015479876160991</v>
       </c>
     </row>
     <row r="24">
@@ -726,7 +726,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>1.462732919254658</v>
+        <v>1.458204334365325</v>
       </c>
     </row>
     <row r="25">
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>5.285714285714286</v>
+        <v>5.284829721362229</v>
       </c>
     </row>
     <row r="26">
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>9.826086956521738</v>
+        <v>9.823529411764707</v>
       </c>
     </row>
     <row r="27">
@@ -757,7 +757,7 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>2.14</t>
+          <t>2.13</t>
         </is>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>36.42546583850932</v>
+        <v>36.42105263157895</v>
       </c>
     </row>
     <row r="29">
@@ -778,7 +778,7 @@
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>1.249130434782609</v>
+        <v>1.248854489164086</v>
       </c>
     </row>
     <row r="30">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>65.63975155279503</v>
+        <v>65.57585139318886</v>
       </c>
     </row>
     <row r="31">
@@ -798,7 +798,7 @@
         </is>
       </c>
       <c r="B31" s="8" t="n">
-        <v>2.108354037267081</v>
+        <v>2.106470588235295</v>
       </c>
     </row>
   </sheetData>
@@ -898,39 +898,39 @@
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C2" s="4" t="n">
         <v>162</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.5031055900621118</v>
+        <v>0.5015479876160991</v>
       </c>
       <c r="F2" s="6" t="n">
-        <v>1.462732919254658</v>
+        <v>1.458204334365325</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>5.285714285714286</v>
+        <v>5.284829721362229</v>
       </c>
       <c r="H2" s="6" t="n">
-        <v>9.826086956521738</v>
+        <v>9.823529411764707</v>
       </c>
       <c r="I2" s="7" t="inlineStr">
         <is>
-          <t>2.14</t>
+          <t>2.13</t>
         </is>
       </c>
       <c r="J2" s="6" t="n">
-        <v>1.249130434782609</v>
+        <v>1.248854489164086</v>
       </c>
       <c r="K2" s="6" t="n">
-        <v>65.63975155279503</v>
+        <v>65.57585139318886</v>
       </c>
       <c r="L2" s="8" t="n">
-        <v>2.108354037267081</v>
+        <v>2.106470588235295</v>
       </c>
     </row>
     <row r="3">
@@ -1050,7 +1050,7 @@
         </is>
       </c>
       <c r="J5" s="6" t="n">
-        <v>4.924590163934426</v>
+        <v>4.924590163934425</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>32.32786885245902</v>
@@ -1128,14 +1128,14 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="5" customWidth="1" min="3" max="3"/>
     <col width="5" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
     <col width="6" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="19" customWidth="1" min="11" max="11"/>
-    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1249,25 +1249,25 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C3" s="4" t="n">
         <v>36</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0.4186046511627907</v>
+        <v>0.4137931034482759</v>
       </c>
       <c r="F3" s="6" t="n">
-        <v>1.174418604651163</v>
+        <v>1.160919540229885</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>5.976744186046512</v>
+        <v>5.96551724137931</v>
       </c>
       <c r="H3" s="6" t="n">
-        <v>10.04651162790698</v>
+        <v>10.03448275862069</v>
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
@@ -1275,13 +1275,13 @@
         </is>
       </c>
       <c r="J3" s="6" t="n">
-        <v>1.233488372093023</v>
+        <v>1.23264367816092</v>
       </c>
       <c r="K3" s="6" t="n">
-        <v>72.06976744186046</v>
+        <v>71.75862068965517</v>
       </c>
       <c r="L3" s="8" t="n">
-        <v>2.263953488372093</v>
+        <v>2.255172413793104</v>
       </c>
     </row>
     <row r="4">
@@ -1506,7 +1506,7 @@
         <v>63.28571428571428</v>
       </c>
       <c r="L3" s="8" t="n">
-        <v>2.024821428571429</v>
+        <v>2.024821428571428</v>
       </c>
     </row>
     <row r="4">
@@ -1558,25 +1558,25 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>16</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.4</v>
+        <v>0.3902439024390244</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.825</v>
+        <v>0.8048780487804879</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>5.225</v>
+        <v>5.219512195121951</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>7.05</v>
+        <v>7.097560975609756</v>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
@@ -1584,13 +1584,13 @@
         </is>
       </c>
       <c r="J5" s="6" t="n">
-        <v>1.223</v>
+        <v>1.221463414634147</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>55.55</v>
+        <v>55.29268292682926</v>
       </c>
       <c r="L5" s="8" t="n">
-        <v>1.90925</v>
+        <v>1.899268292682927</v>
       </c>
     </row>
     <row r="6">
@@ -1626,7 +1626,7 @@
         </is>
       </c>
       <c r="J6" s="6" t="n">
-        <v>5.148285714285715</v>
+        <v>5.148285714285714</v>
       </c>
       <c r="K6" s="6" t="n">
         <v>34.6</v>
@@ -1842,7 +1842,7 @@
         <v>25.625</v>
       </c>
       <c r="L11" s="8" t="n">
-        <v>0.85625</v>
+        <v>0.8562500000000001</v>
       </c>
     </row>
     <row r="12">
@@ -2046,7 +2046,7 @@
         </is>
       </c>
       <c r="J16" s="6" t="n">
-        <v>5.050000000000001</v>
+        <v>5.05</v>
       </c>
       <c r="K16" s="6" t="n">
         <v>16.25</v>
@@ -2823,7 +2823,7 @@
         <v>64.09090909090909</v>
       </c>
       <c r="L3" s="8" t="n">
-        <v>2.045636363636364</v>
+        <v>2.045636363636363</v>
       </c>
     </row>
     <row r="4">
@@ -2875,25 +2875,25 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>16</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.4</v>
+        <v>0.3902439024390244</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.825</v>
+        <v>0.8048780487804879</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>5.225</v>
+        <v>5.219512195121951</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>7.05</v>
+        <v>7.097560975609756</v>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
@@ -2901,13 +2901,13 @@
         </is>
       </c>
       <c r="J5" s="6" t="n">
-        <v>1.223</v>
+        <v>1.221463414634147</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>55.55</v>
+        <v>55.29268292682926</v>
       </c>
       <c r="L5" s="8" t="n">
-        <v>1.90925</v>
+        <v>1.899268292682927</v>
       </c>
     </row>
     <row r="6">
@@ -3308,7 +3308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V406"/>
+  <dimension ref="A1:V407"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -35847,8 +35847,88 @@
         </is>
       </c>
     </row>
+    <row r="407">
+      <c r="A407" s="7" t="inlineStr">
+        <is>
+          <t>2026-01-05 23:21:47</t>
+        </is>
+      </c>
+      <c r="B407" s="7" t="inlineStr">
+        <is>
+          <t>ランク(ソロ/デュオ)</t>
+        </is>
+      </c>
+      <c r="C407" s="12" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D407" s="7" t="inlineStr">
+        <is>
+          <t>SUP</t>
+        </is>
+      </c>
+      <c r="E407" s="7" t="inlineStr">
+        <is>
+          <t>ジャンナ</t>
+        </is>
+      </c>
+      <c r="F407" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G407" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H407" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="I407" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J407" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="K407" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="L407" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="M407" s="6" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="N407" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="O407" s="8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="P407" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q407" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="R407" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="S407" s="11" t="n">
+        <v>6751</v>
+      </c>
+      <c r="T407" s="11" t="n">
+        <v>2219</v>
+      </c>
+      <c r="U407" s="6" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="V407" s="7" t="inlineStr">
+        <is>
+          <t>JP1_556572228</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:V406"/>
+  <autoFilter ref="A1:V407"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -35859,7 +35939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P406"/>
+  <dimension ref="A1:P407"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -61072,8 +61152,70 @@
         </is>
       </c>
     </row>
+    <row r="407">
+      <c r="A407" s="13" t="inlineStr">
+        <is>
+          <t>2026-01-05 23:21:47</t>
+        </is>
+      </c>
+      <c r="B407" s="13" t="inlineStr">
+        <is>
+          <t>ランク</t>
+        </is>
+      </c>
+      <c r="C407" s="13" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D407" s="13" t="inlineStr">
+        <is>
+          <t>SUP</t>
+        </is>
+      </c>
+      <c r="E407" s="13" t="inlineStr">
+        <is>
+          <t>ジャンナ</t>
+        </is>
+      </c>
+      <c r="F407" s="13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G407" s="13" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H407" s="13" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="I407" s="13" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="J407" s="13" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="K407" s="14" t="inlineStr"/>
+      <c r="L407" s="14" t="inlineStr"/>
+      <c r="M407" s="14" t="inlineStr"/>
+      <c r="N407" s="14" t="inlineStr"/>
+      <c r="O407" s="14" t="inlineStr"/>
+      <c r="P407" s="13" t="inlineStr">
+        <is>
+          <t>JP1_556572228</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P406"/>
+  <autoFilter ref="A1:P407"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>